<commit_message>
docs(test): Complete final SIT test cases for collateral and loan
</commit_message>
<xml_diff>
--- a/5. Kiểm thử/SIT/SIT_ETL_TestCases.xlsx
+++ b/5. Kiểm thử/SIT/SIT_ETL_TestCases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Công việc\1. Dự án Gỗ Minh Long\5. Kiểm thử\SIT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF4C3A51-8385-4B89-9F0F-E7E8FD11F462}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF7EA52F-0C2D-4A61-9C0C-3489B621CDAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="164">
   <si>
     <t>Case ID</t>
   </si>
@@ -503,9 +503,6 @@
   </si>
   <si>
     <t>Hop_dong_tien_gui.xlsx</t>
-  </si>
-  <si>
-    <t>[ ] Pending</t>
   </si>
   <si>
     <t>Chạy SQL: SELECT _id, COUNT(*) FROM silver.fact_cashflow GROUP BY _id HAVING COUNT(*) &gt; 1;;</t>
@@ -883,14 +880,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J41"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="25.6640625" customWidth="1"/>
-    <col min="5" max="5" width="73.44140625" customWidth="1"/>
-    <col min="7" max="7" width="35.5546875" customWidth="1"/>
+    <col min="3" max="3" width="6.140625" customWidth="1"/>
+    <col min="4" max="4" width="25.7109375" customWidth="1"/>
+    <col min="5" max="5" width="3.42578125" customWidth="1"/>
+    <col min="7" max="7" width="37.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -922,7 +920,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -945,13 +943,13 @@
         <v>143</v>
       </c>
       <c r="I2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="J2">
         <v>295</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -974,13 +972,13 @@
         <v>143</v>
       </c>
       <c r="I3" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -1003,13 +1001,13 @@
         <v>144</v>
       </c>
       <c r="I4" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="J4">
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -1032,13 +1030,13 @@
         <v>144</v>
       </c>
       <c r="I5" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -1061,13 +1059,13 @@
         <v>145</v>
       </c>
       <c r="I6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="J6">
         <v>43</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>15</v>
       </c>
@@ -1090,13 +1088,13 @@
         <v>145</v>
       </c>
       <c r="I7" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -1119,13 +1117,13 @@
         <v>146</v>
       </c>
       <c r="I8" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="J8">
         <v>2688</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>17</v>
       </c>
@@ -1148,13 +1146,13 @@
         <v>146</v>
       </c>
       <c r="I9" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="J9">
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>18</v>
       </c>
@@ -1177,13 +1175,13 @@
         <v>147</v>
       </c>
       <c r="I10" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="J10">
         <v>145086</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>19</v>
       </c>
@@ -1206,13 +1204,13 @@
         <v>147</v>
       </c>
       <c r="I11" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="J11">
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>20</v>
       </c>
@@ -1235,13 +1233,13 @@
         <v>148</v>
       </c>
       <c r="I12" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="J12">
         <v>147</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>21</v>
       </c>
@@ -1264,13 +1262,13 @@
         <v>148</v>
       </c>
       <c r="I13" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="J13">
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>22</v>
       </c>
@@ -1293,13 +1291,13 @@
         <v>149</v>
       </c>
       <c r="I14" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="J14">
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>23</v>
       </c>
@@ -1322,13 +1320,13 @@
         <v>149</v>
       </c>
       <c r="I15" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="J15">
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>24</v>
       </c>
@@ -1351,13 +1349,13 @@
         <v>150</v>
       </c>
       <c r="I16" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="J16">
         <v>16447</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>25</v>
       </c>
@@ -1380,13 +1378,13 @@
         <v>150</v>
       </c>
       <c r="I17" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="J17">
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>26</v>
       </c>
@@ -1409,13 +1407,13 @@
         <v>151</v>
       </c>
       <c r="I18" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="J18">
         <v>28886</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>27</v>
       </c>
@@ -1438,13 +1436,13 @@
         <v>151</v>
       </c>
       <c r="I19" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="J19">
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>28</v>
       </c>
@@ -1467,13 +1465,13 @@
         <v>152</v>
       </c>
       <c r="I20" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="J20">
         <v>252</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>29</v>
       </c>
@@ -1496,13 +1494,13 @@
         <v>152</v>
       </c>
       <c r="I21" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="J21">
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>30</v>
       </c>
@@ -1525,13 +1523,13 @@
         <v>153</v>
       </c>
       <c r="I22" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="J22">
         <v>1680</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>31</v>
       </c>
@@ -1554,13 +1552,13 @@
         <v>153</v>
       </c>
       <c r="I23" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="J23">
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>32</v>
       </c>
@@ -1574,7 +1572,7 @@
         <v>64</v>
       </c>
       <c r="E24" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F24" t="s">
         <v>132</v>
@@ -1583,13 +1581,13 @@
         <v>154</v>
       </c>
       <c r="I24" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="J24">
         <v>251861</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>33</v>
       </c>
@@ -1612,13 +1610,13 @@
         <v>154</v>
       </c>
       <c r="I25" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="J25">
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>34</v>
       </c>
@@ -1641,13 +1639,13 @@
         <v>155</v>
       </c>
       <c r="I26" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="J26">
         <v>34</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>35</v>
       </c>
@@ -1670,13 +1668,13 @@
         <v>155</v>
       </c>
       <c r="I27" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="J27">
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>36</v>
       </c>
@@ -1699,13 +1697,13 @@
         <v>155</v>
       </c>
       <c r="I28" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="J28">
         <v>7</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>37</v>
       </c>
@@ -1728,13 +1726,13 @@
         <v>155</v>
       </c>
       <c r="I29" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="J29">
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>38</v>
       </c>
@@ -1757,13 +1755,13 @@
         <v>156</v>
       </c>
       <c r="I30" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="J30">
         <v>42</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>39</v>
       </c>
@@ -1786,13 +1784,13 @@
         <v>156</v>
       </c>
       <c r="I31" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="J31">
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>40</v>
       </c>
@@ -1815,13 +1813,13 @@
         <v>157</v>
       </c>
       <c r="I32" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="J32">
         <v>6589</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>41</v>
       </c>
@@ -1844,13 +1842,13 @@
         <v>157</v>
       </c>
       <c r="I33" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="J33">
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>42</v>
       </c>
@@ -1873,13 +1871,13 @@
         <v>158</v>
       </c>
       <c r="I34" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="J34">
         <v>8042</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>43</v>
       </c>
@@ -1902,13 +1900,13 @@
         <v>158</v>
       </c>
       <c r="I35" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="J35">
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>44</v>
       </c>
@@ -1931,13 +1929,13 @@
         <v>159</v>
       </c>
       <c r="I36" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="J36">
         <v>12471</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>45</v>
       </c>
@@ -1960,13 +1958,13 @@
         <v>159</v>
       </c>
       <c r="I37" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="J37">
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>46</v>
       </c>
@@ -1989,13 +1987,13 @@
         <v>155</v>
       </c>
       <c r="I38" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="J38">
         <v>258</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>47</v>
       </c>
@@ -2018,13 +2016,13 @@
         <v>155</v>
       </c>
       <c r="I39" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="J39">
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>48</v>
       </c>
@@ -2047,13 +2045,13 @@
         <v>160</v>
       </c>
       <c r="I40" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="J40">
         <v>72</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>49</v>
       </c>
@@ -2067,7 +2065,7 @@
         <v>72</v>
       </c>
       <c r="E41" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F41" t="s">
         <v>142</v>
@@ -2076,7 +2074,7 @@
         <v>160</v>
       </c>
       <c r="I41" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="J41">
         <v>0</v>

</xml_diff>